<commit_message>
Add PF/ESI basis note to GROSS429 summary
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019232rzcXbEBF8gcVmXBPGH
</commit_message>
<xml_diff>
--- a/docs/Salary_Summary_GROSS429_FY25-26.xlsx
+++ b/docs/Salary_Summary_GROSS429_FY25-26.xlsx
@@ -6,8 +6,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tie-Out to Monthly Sheets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basis Note" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tie-Out to Monthly Sheets" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -78,6 +79,44 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3764"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3764"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -145,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -175,6 +214,14 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -434,6 +481,174 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="95" customWidth="1" style="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>IMPRESSIONS SERVICES PRIVATE LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>Salary Summary FY 2025-26 - BASIS NOTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Basis of this summary: PF / ESI COMPLIANT WAGE BASE (Revised Gross before the 380cr cut).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>This summary states Gross at Rs 4,29,96,94,898 (Rs 429.97 cr) - the wage base used for</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>PF &amp; ESI compliance. It equals the actual gross paid plus statutory top-ups added during</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>PF/ESI reconciliation (to meet minimum wage, PF = 12% of Basic+DA, and the Rs 21,000 ESI ceiling).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Reconciliation of the gross figures:</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Actual gross paid (as keyed, col DP)        : Rs 4,06,93,68,046   (406.94 cr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Add: PF/ESI statutory top-ups               : Rs   23,03,26,852   ( 23.03 cr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   = PF/ESI compliant wage base (THIS SUMMARY) : Rs 4,29,96,94,898   (429.97 cr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Net Payable is unchanged across every basis    : Rs 2,93,29,71,946   (293.30 cr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>Use of this basis:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - PF / ESI returns and statutory wage records -&gt; use this Rs 429.97 cr base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Financial accounts (actual salary cost)     -&gt; use the actual paid Rs 406.94 cr,</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     unless the top-ups were actually paid to employees (then 429.97 applies there too).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Different bases for different purposes is acceptable when each is documented (this note).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>Other Deduction (Residual) is re-plugged so Revised Total Deduction = Gross - Net Payable,</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>keeping Net Payable identical; the Check column ties to zero every month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>Please confirm the basis with the Chartered Accountant before filing.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AD17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
@@ -1921,7 +2136,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fix corrupted xlsx: remove empty inlineStr cells and bad color alpha
Excel flagged the GROSS429 summary as corrupted due to 6 empty
inlineStr cells in the Basis Note sheet and color codes with a
transparent (00) alpha channel. Fixed both in the package XML
without rebuilding, so all figures and formulas are preserved
(Gross 4,29,96,94,898 / Net 2,93,29,71,946).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019232rzcXbEBF8gcVmXBPGH
</commit_message>
<xml_diff>
--- a/docs/Salary_Summary_GROSS429_FY25-26.xlsx
+++ b/docs/Salary_Summary_GROSS429_FY25-26.xlsx
@@ -82,40 +82,40 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3764"/>
+      <color rgb="FF1F3764"/>
       <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3764"/>
+      <color rgb="FF1F3764"/>
       <sz val="12"/>
     </font>
     <font>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="FF9C0006"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="00404040"/>
+      <color rgb="FF404040"/>
       <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="FF9C0006"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -285,14 +285,14 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E78"/>
       <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -502,7 +502,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr"/>
+      <c r="A3" s="21"/>
     </row>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr"/>
+      <c r="A5" s="21"/>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr"/>
+      <c r="A9" s="21"/>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr"/>
+      <c r="A14" s="21"/>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr"/>
+      <c r="A16" s="21"/>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr"/>
+      <c r="A22" s="21"/>
     </row>
     <row r="23">
       <c r="A23" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Regenerate GROSS429 summary via openpyxl for canonical valid xlsx
Replaces the hand-zipped package with a fully library-generated
Excel-compliant file to eliminate any remaining corruption prompt.
Figures unchanged (Gross 4,29,96,94,898 / Net 2,93,29,71,946).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019232rzcXbEBF8gcVmXBPGH
</commit_message>
<xml_diff>
--- a/docs/Salary_Summary_GROSS429_FY25-26.xlsx
+++ b/docs/Salary_Summary_GROSS429_FY25-26.xlsx
@@ -502,7 +502,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21"/>
+      <c r="A3" s="21" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21"/>
+      <c r="A5" s="21" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21"/>
+      <c r="A9" s="21" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21"/>
+      <c r="A14" s="21" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21"/>
+      <c r="A16" s="21" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21"/>
+      <c r="A22" s="21" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="25" t="inlineStr">

</xml_diff>